<commit_message>
Added sample data for test run without need to download; Added figures; fixed environment
</commit_message>
<xml_diff>
--- a/cCRE_based_analysis/data/supplementary/supplementary_table_enriched_tfs_active_vs_not_significant.xlsx
+++ b/cCRE_based_analysis/data/supplementary/supplementary_table_enriched_tfs_active_vs_not_significant.xlsx
@@ -70,21 +70,21 @@
     <t>SALL4</t>
   </si>
   <si>
+    <t>JDP2</t>
+  </si>
+  <si>
+    <t>ZNF7</t>
+  </si>
+  <si>
     <t>ZNF502</t>
   </si>
   <si>
-    <t>ZNF7</t>
+    <t>ZNF704</t>
   </si>
   <si>
     <t>ZNF430</t>
   </si>
   <si>
-    <t>ZNF704</t>
-  </si>
-  <si>
-    <t>JDP2</t>
-  </si>
-  <si>
     <t>ZNF432</t>
   </si>
   <si>
@@ -118,12 +118,12 @@
     <t>ZNF256</t>
   </si>
   <si>
+    <t>HOMEZ</t>
+  </si>
+  <si>
     <t>ARID3B</t>
   </si>
   <si>
-    <t>HOMEZ</t>
-  </si>
-  <si>
     <t>ZNF740</t>
   </si>
   <si>
@@ -151,24 +151,24 @@
     <t>KAT2B</t>
   </si>
   <si>
+    <t>ZNF93</t>
+  </si>
+  <si>
     <t>RUVBL1</t>
   </si>
   <si>
-    <t>ZNF93</t>
-  </si>
-  <si>
     <t>ZNF765</t>
   </si>
   <si>
+    <t>ZNF701</t>
+  </si>
+  <si>
+    <t>SAFB</t>
+  </si>
+  <si>
     <t>ZNF302</t>
   </si>
   <si>
-    <t>SAFB</t>
-  </si>
-  <si>
-    <t>ZNF701</t>
-  </si>
-  <si>
     <t>FANCL</t>
   </si>
   <si>
@@ -193,12 +193,12 @@
     <t>ZBTB14</t>
   </si>
   <si>
+    <t>DR1</t>
+  </si>
+  <si>
     <t>SNAPC1</t>
   </si>
   <si>
-    <t>DR1</t>
-  </si>
-  <si>
     <t>OGT</t>
   </si>
   <si>
@@ -475,12 +475,12 @@
     <t>KLF7</t>
   </si>
   <si>
+    <t>PHF19</t>
+  </si>
+  <si>
     <t>ARID5B</t>
   </si>
   <si>
-    <t>PHF19</t>
-  </si>
-  <si>
     <t>ZNF142</t>
   </si>
   <si>
@@ -1099,15 +1099,15 @@
     <t>ZNF143</t>
   </si>
   <si>
+    <t>ZNF362</t>
+  </si>
+  <si>
     <t>CCAR2</t>
   </si>
   <si>
     <t>CBX3</t>
   </si>
   <si>
-    <t>ZNF362</t>
-  </si>
-  <si>
     <t>KDM3A</t>
   </si>
   <si>
@@ -1132,10 +1132,10 @@
     <t>MYNN</t>
   </si>
   <si>
+    <t>NFKBIZ</t>
+  </si>
+  <si>
     <t>SOX4</t>
-  </si>
-  <si>
-    <t>NFKBIZ</t>
   </si>
   <si>
     <t>FEZF1</t>
@@ -1544,8 +1544,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1561,7 +1569,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1569,12 +1577,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1873,40 +1899,40 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7279,13 +7305,13 @@
         <v>0.0001445803698057228</v>
       </c>
       <c r="D143">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E143">
         <v>22</v>
       </c>
       <c r="F143">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G143" t="s">
         <v>507</v>
@@ -7317,13 +7343,13 @@
         <v>0.0001445803698057228</v>
       </c>
       <c r="D144">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E144">
         <v>22</v>
       </c>
       <c r="F144">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G144" t="s">
         <v>507</v>
@@ -15183,13 +15209,13 @@
         <v>0.006659669281280164</v>
       </c>
       <c r="D351">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E351">
         <v>38</v>
       </c>
       <c r="F351">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G351" t="s">
         <v>507</v>
@@ -15221,13 +15247,13 @@
         <v>0.006659669281280164</v>
       </c>
       <c r="D352">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E352">
         <v>38</v>
       </c>
       <c r="F352">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G352" t="s">
         <v>507</v>
@@ -15601,13 +15627,13 @@
         <v>0.001046316999309153</v>
       </c>
       <c r="D362">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="E362">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F362">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="G362" t="s">
         <v>507</v>
@@ -15639,13 +15665,13 @@
         <v>0.001046316999309153</v>
       </c>
       <c r="D363">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="E363">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F363">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="G363" t="s">
         <v>507</v>

</xml_diff>